<commit_message>
Add PO tracking, dashboard PO chart, and history.html PO assignment fixes
- Add net_price/currency to po_data, show PO price + "Deliv. Compl." filtering in history.html PO dropdowns and dashboard PO balance chart
- Add bulk PO-assign, allow production dept to assign PO on history.html
- Add PO Balance chart (stacked, per-PO received vs pending) and convert daily plan-vs-actual chart to columns
- Fix email-preview-supplier.html stuck-spinner bug, populate From: with sender email, confirm-popup before send
- Consolidate Bioligo IH200 -> Bioligo IMO across code and DB
- Auto-apply history.html filters without needing the "กรอง" button
- Misc: cache-busting on generated navigation URLs, requirement.md updates
</commit_message>
<xml_diff>
--- a/PO_matcall.XLSX
+++ b/PO_matcall.XLSX
@@ -166,7 +166,7 @@
     <t>0010027535</t>
   </si>
   <si>
-    <t>แปซิฟิก ชูการ์ คอร์ปอเรชั่น</t>
+    <t>Pacific Sugar Corporation Limited</t>
   </si>
   <si>
     <t>0105090136</t>
@@ -487,7 +487,7 @@
     <t>0010006985</t>
   </si>
   <si>
-    <t>ดับเบิ้ลยูจีซี</t>
+    <t>WGC CO.,LTD.</t>
   </si>
   <si>
     <t>0105104205</t>
@@ -9313,10 +9313,10 @@
         <v>195000.000</v>
       </c>
       <c r="W72" s="3">
-        <v>99950.000</v>
+        <v>129990.000</v>
       </c>
       <c r="X72" s="3">
-        <v>95050.000</v>
+        <v>65010.000</v>
       </c>
       <c r="Y72" t="s">
         <v>15</v>
@@ -9346,7 +9346,7 @@
         <v>2827500.00</v>
       </c>
       <c r="AH72" s="5">
-        <v>1449275.00</v>
+        <v>1884855.00</v>
       </c>
       <c r="AI72" t="s">
         <v>9</v>
@@ -10119,10 +10119,10 @@
         <v>260000.000</v>
       </c>
       <c r="W79" s="3">
-        <v>229970.000</v>
+        <v>260000.000</v>
       </c>
       <c r="X79" s="3">
-        <v>30030.000</v>
+        <v>0.000</v>
       </c>
       <c r="Y79" t="s">
         <v>15</v>
@@ -10152,10 +10152,10 @@
         <v>3770000.00</v>
       </c>
       <c r="AH79" s="5">
-        <v>3334565.00</v>
+        <v>3770000.00</v>
       </c>
       <c r="AI79" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="AJ79" t="s">
         <v>9</v>
@@ -10929,10 +10929,10 @@
         <v>60000.000</v>
       </c>
       <c r="W86" s="3">
-        <v>50000.000</v>
+        <v>60000.000</v>
       </c>
       <c r="X86" s="3">
-        <v>10000.000</v>
+        <v>0.000</v>
       </c>
       <c r="Y86" t="s">
         <v>15</v>
@@ -10962,10 +10962,10 @@
         <v>945000.00</v>
       </c>
       <c r="AH86" s="5">
-        <v>787500.00</v>
+        <v>945000.00</v>
       </c>
       <c r="AI86" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="AJ86" t="s">
         <v>9</v>
@@ -11045,15 +11045,17 @@
         <v>140000.000</v>
       </c>
       <c r="W87" s="3">
-        <v>0.000</v>
+        <v>15010.000</v>
       </c>
       <c r="X87" s="3">
-        <v>140000.000</v>
+        <v>124990.000</v>
       </c>
       <c r="Y87" t="s">
         <v>15</v>
       </c>
-      <c r="Z87" s="2"/>
+      <c r="Z87" s="2">
+        <v>46218</v>
+      </c>
       <c r="AA87" s="2">
         <v>46146</v>
       </c>
@@ -11061,7 +11063,7 @@
         <v>46143</v>
       </c>
       <c r="AC87" s="4">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="AD87" s="5">
         <v>15.75</v>
@@ -11076,7 +11078,7 @@
         <v>2205000.00</v>
       </c>
       <c r="AH87" s="5">
-        <v>0.00</v>
+        <v>236407.50</v>
       </c>
       <c r="AI87" t="s">
         <v>9</v>
@@ -11739,10 +11741,10 @@
         <v>530000.000</v>
       </c>
       <c r="W93" s="3">
-        <v>360340.000</v>
+        <v>341640.000</v>
       </c>
       <c r="X93" s="3">
-        <v>0.000</v>
+        <v>188360.000</v>
       </c>
       <c r="Y93" t="s">
         <v>15</v>
@@ -11772,10 +11774,10 @@
         <v>3015700.00</v>
       </c>
       <c r="AH93" s="5">
-        <v>2050334.60</v>
+        <v>1943931.60</v>
       </c>
       <c r="AI93" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AJ93" t="s">
         <v>9</v>
@@ -15327,10 +15329,10 @@
         <v>300000.000</v>
       </c>
       <c r="W124" s="3">
-        <v>209720.000</v>
+        <v>239700.000</v>
       </c>
       <c r="X124" s="3">
-        <v>90280.000</v>
+        <v>60300.000</v>
       </c>
       <c r="Y124" t="s">
         <v>15</v>
@@ -15360,7 +15362,7 @@
         <v>4593000.00</v>
       </c>
       <c r="AH124" s="5">
-        <v>3210813.20</v>
+        <v>3669807.00</v>
       </c>
       <c r="AI124" t="s">
         <v>9</v>
@@ -15671,15 +15673,17 @@
         <v>22500.000</v>
       </c>
       <c r="W127" s="3">
+        <v>22500.000</v>
+      </c>
+      <c r="X127" s="3">
         <v>0.000</v>
-      </c>
-      <c r="X127" s="3">
-        <v>22500.000</v>
       </c>
       <c r="Y127" t="s">
         <v>15</v>
       </c>
-      <c r="Z127" s="2"/>
+      <c r="Z127" s="2">
+        <v>46219</v>
+      </c>
       <c r="AA127" s="2">
         <v>46203</v>
       </c>
@@ -15687,7 +15691,7 @@
         <v>46204</v>
       </c>
       <c r="AC127" s="4">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="AD127" s="5">
         <v>15.38</v>
@@ -15702,10 +15706,10 @@
         <v>346050.00</v>
       </c>
       <c r="AH127" s="5">
-        <v>0.00</v>
+        <v>346050.00</v>
       </c>
       <c r="AI127" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="AJ127" t="s">
         <v>9</v>
@@ -15785,10 +15789,10 @@
         <v>40000.000</v>
       </c>
       <c r="W128" s="3">
-        <v>29980.000</v>
+        <v>37460.000</v>
       </c>
       <c r="X128" s="3">
-        <v>10020.000</v>
+        <v>2540.000</v>
       </c>
       <c r="Y128" t="s">
         <v>15</v>
@@ -15818,7 +15822,7 @@
         <v>615200.00</v>
       </c>
       <c r="AH128" s="5">
-        <v>461092.40</v>
+        <v>576134.80</v>
       </c>
       <c r="AI128" t="s">
         <v>9</v>
@@ -16479,15 +16483,17 @@
         <v>550000.000</v>
       </c>
       <c r="W134" s="3">
-        <v>0.000</v>
+        <v>76590.000</v>
       </c>
       <c r="X134" s="3">
-        <v>550000.000</v>
+        <v>473410.000</v>
       </c>
       <c r="Y134" t="s">
         <v>15</v>
       </c>
-      <c r="Z134" s="2"/>
+      <c r="Z134" s="2">
+        <v>46205</v>
+      </c>
       <c r="AA134" s="2">
         <v>46216</v>
       </c>
@@ -16495,7 +16501,7 @@
         <v>46204</v>
       </c>
       <c r="AC134" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD134" s="5">
         <v>5.85</v>
@@ -16510,7 +16516,7 @@
         <v>3217500.00</v>
       </c>
       <c r="AH134" s="5">
-        <v>0.00</v>
+        <v>448051.50</v>
       </c>
       <c r="AI134" t="s">
         <v>9</v>
@@ -16593,15 +16599,17 @@
         <v>550000.000</v>
       </c>
       <c r="W135" s="3">
-        <v>0.000</v>
+        <v>76130.000</v>
       </c>
       <c r="X135" s="3">
-        <v>550000.000</v>
+        <v>473870.000</v>
       </c>
       <c r="Y135" t="s">
         <v>15</v>
       </c>
-      <c r="Z135" s="2"/>
+      <c r="Z135" s="2">
+        <v>46210</v>
+      </c>
       <c r="AA135" s="2">
         <v>46216</v>
       </c>
@@ -16609,7 +16617,7 @@
         <v>46204</v>
       </c>
       <c r="AC135" s="4">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD135" s="5">
         <v>5.85</v>
@@ -16624,7 +16632,7 @@
         <v>3217500.00</v>
       </c>
       <c r="AH135" s="5">
-        <v>0.00</v>
+        <v>445360.50</v>
       </c>
       <c r="AI135" t="s">
         <v>9</v>

</xml_diff>